<commit_message>
refactor: update year selection text and enhance acceptance year logic
</commit_message>
<xml_diff>
--- a/translations/welsh-translations/xlsx/21-producer-prns-prn-choose-year.xlsx
+++ b/translations/welsh-translations/xlsx/21-producer-prns-prn-choose-year.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>Translator notes</t>
   </si>
@@ -58,13 +58,7 @@
     <t>prns.chooseYear.heading</t>
   </si>
   <si>
-    <t>Which year do you want to accept this {{type}} into?</t>
-  </si>
-  <si>
-    <t>prns.chooseYear.hint</t>
-  </si>
-  <si>
-    <t>Select the obligation year this December waste will count towards.</t>
+    <t>Which year’s recycling obligations do you want to accept this {{type}} towards?</t>
   </si>
   <si>
     <t>prns.chooseYear.continueButton</t>
@@ -475,7 +469,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" hidden="1" customWidth="1"/>
@@ -606,28 +600,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:F10"/>
+  <autoFilter ref="A5:F9"/>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="D2:F2"/>

</xml_diff>